<commit_message>
fixed computation methods of netflow
</commit_message>
<xml_diff>
--- a/xlsxReports/cpu_netflow_men_report.xlsx
+++ b/xlsxReports/cpu_netflow_men_report.xlsx
@@ -330,184 +330,184 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="60"/>
                 <c:pt idx="0">
-                  <c:v>163</c:v>
+                  <c:v>141</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>168</c:v>
+                  <c:v>134</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>159</c:v>
+                  <c:v>127</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>133</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>71.40000000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>143</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>162</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>154</c:v>
-                </c:pt>
                 <c:pt idx="6">
-                  <c:v>162</c:v>
+                  <c:v>113</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>178</c:v>
+                  <c:v>144</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>168</c:v>
+                  <c:v>137</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>162</c:v>
+                  <c:v>117</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>168</c:v>
+                  <c:v>144</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>171</c:v>
+                  <c:v>126</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>159</c:v>
+                  <c:v>126</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>175</c:v>
+                  <c:v>153</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>168</c:v>
+                  <c:v>141</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>168</c:v>
+                  <c:v>143</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>165</c:v>
+                  <c:v>134</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>171</c:v>
+                  <c:v>134</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>175</c:v>
+                  <c:v>144</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>171</c:v>
+                  <c:v>141</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>171</c:v>
+                  <c:v>137</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>168</c:v>
+                  <c:v>134</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>171</c:v>
+                  <c:v>127</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>162</c:v>
+                  <c:v>141</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>156</c:v>
+                  <c:v>130</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>165</c:v>
+                  <c:v>137</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>165</c:v>
+                  <c:v>144</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>165</c:v>
+                  <c:v>75.8</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>162</c:v>
+                  <c:v>114</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>165</c:v>
+                  <c:v>131</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>165</c:v>
+                  <c:v>140</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>165</c:v>
+                  <c:v>107</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>165</c:v>
+                  <c:v>96.59999999999999</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>162</c:v>
+                  <c:v>66.59999999999999</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>181</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="35">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>137</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>144</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>141</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>131</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>151</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>92.8</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>143</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>141</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>78.5</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>78.5</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>82.09999999999999</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>141</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>60.7</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>78.5</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>67.8</c:v>
+                </c:pt>
+                <c:pt idx="56">
                   <c:v>153</c:v>
                 </c:pt>
-                <c:pt idx="36">
-                  <c:v>178</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>165</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>175</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>175</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>165</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>157</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>175</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>175</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>181</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>165</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>165</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>168</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>159</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>168</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>196</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>165</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>162</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>168</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>171</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>184</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>159</c:v>
-                </c:pt>
                 <c:pt idx="57">
-                  <c:v>171</c:v>
+                  <c:v>82.7</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>171</c:v>
+                  <c:v>120</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>159</c:v>
+                  <c:v>64.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -829,184 +829,184 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="60"/>
                 <c:pt idx="0">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-110393</c:v>
+                  <c:v>66</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-110393</c:v>
+                  <c:v>140</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-110393</c:v>
+                  <c:v>94</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-110393</c:v>
+                  <c:v>367</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-110393</c:v>
+                  <c:v>140</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-110393</c:v>
+                  <c:v>5323</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-110393</c:v>
+                  <c:v>66</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>-110393</c:v>
+                  <c:v>525</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>-110393</c:v>
+                  <c:v>1558</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>-110393</c:v>
+                  <c:v>433</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1222,184 +1222,184 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="60"/>
                 <c:pt idx="0">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-110393</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-110393</c:v>
+                  <c:v>148</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-110393</c:v>
+                  <c:v>538</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-110393</c:v>
+                  <c:v>259</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-110393</c:v>
+                  <c:v>116</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-110393</c:v>
+                  <c:v>1337</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-110393</c:v>
+                  <c:v>197</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>-110393</c:v>
+                  <c:v>2960</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>-110393</c:v>
+                  <c:v>10711</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>-110393</c:v>
+                  <c:v>748</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>-110393</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1615,184 +1615,184 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="60"/>
                 <c:pt idx="0">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-220786</c:v>
+                  <c:v>115</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-220786</c:v>
+                  <c:v>288</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-220786</c:v>
+                  <c:v>538</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-220786</c:v>
+                  <c:v>94</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-220786</c:v>
+                  <c:v>626</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-220786</c:v>
+                  <c:v>256</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-220786</c:v>
+                  <c:v>6660</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-220786</c:v>
+                  <c:v>263</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>-220786</c:v>
+                  <c:v>3485</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>-220786</c:v>
+                  <c:v>12269</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>-220786</c:v>
+                  <c:v>1181</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>-220786</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2114,184 +2114,184 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="60"/>
                 <c:pt idx="0">
-                  <c:v>12.1</c:v>
+                  <c:v>7.6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12.1</c:v>
+                  <c:v>7.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12.1</c:v>
+                  <c:v>7.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>12.1</c:v>
+                  <c:v>7.6</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12.1</c:v>
+                  <c:v>7.6</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>12.6</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>12.1</c:v>
+                  <c:v>7.4</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>12.1</c:v>
+                  <c:v>7.4</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>12.1</c:v>
+                  <c:v>7.4</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>12.1</c:v>
+                  <c:v>7.4</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>12.1</c:v>
+                  <c:v>7.4</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>12.1</c:v>
+                  <c:v>7.4</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>12.1</c:v>
+                  <c:v>7.4</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>12.1</c:v>
+                  <c:v>7.4</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>12.1</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>12.1</c:v>
+                  <c:v>7.8</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>12.1</c:v>
+                  <c:v>7.8</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>12.2</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>12.2</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>12.2</c:v>
+                  <c:v>7.8</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>12.1</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>12.1</c:v>
+                  <c:v>7.8</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>12.1</c:v>
+                  <c:v>7.8</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>12.1</c:v>
+                  <c:v>8.9</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>12.1</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>12.1</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>12.1</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>12.1</c:v>
+                  <c:v>8.6</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>12.1</c:v>
+                  <c:v>8.6</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>12.1</c:v>
+                  <c:v>8.699999999999999</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>12.1</c:v>
+                  <c:v>9.4</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>12.1</c:v>
+                  <c:v>9.199999999999999</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>12.1</c:v>
+                  <c:v>8.699999999999999</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>12.1</c:v>
+                  <c:v>8.699999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2613,184 +2613,184 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="60"/>
                 <c:pt idx="0">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>99</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3316,7 +3316,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>163</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -3324,7 +3324,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>168</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -3332,7 +3332,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>159</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -3340,7 +3340,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>143</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -3348,7 +3348,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>162</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -3356,7 +3356,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>154</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -3364,7 +3364,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>162</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -3372,7 +3372,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>178</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -3380,7 +3380,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>168</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -3388,7 +3388,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>162</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -3396,7 +3396,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>168</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -3404,7 +3404,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>171</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -3412,7 +3412,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>159</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -3420,7 +3420,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>175</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -3428,7 +3428,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>168</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -3436,7 +3436,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>168</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -3444,7 +3444,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>165</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -3452,7 +3452,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>171</v>
+        <v>134</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -3460,7 +3460,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>175</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -3468,7 +3468,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>171</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -3476,7 +3476,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>171</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -3484,7 +3484,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>168</v>
+        <v>134</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -3492,7 +3492,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>171</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -3500,7 +3500,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>162</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -3508,7 +3508,7 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>156</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -3516,7 +3516,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>165</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -3524,7 +3524,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>165</v>
+        <v>144</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -3532,7 +3532,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>165</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -3540,7 +3540,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>162</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -3548,7 +3548,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>165</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -3556,7 +3556,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>165</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -3564,7 +3564,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>165</v>
+        <v>107</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -3572,7 +3572,7 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>165</v>
+        <v>96.59999999999999</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -3580,7 +3580,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>162</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -3588,7 +3588,7 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>181</v>
+        <v>150</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -3596,7 +3596,7 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -3604,7 +3604,7 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>178</v>
+        <v>137</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -3612,7 +3612,7 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>165</v>
+        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -3620,7 +3620,7 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>175</v>
+        <v>144</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -3628,7 +3628,7 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>175</v>
+        <v>141</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -3636,7 +3636,7 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>165</v>
+        <v>131</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -3644,7 +3644,7 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -3652,7 +3652,7 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>175</v>
+        <v>155</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -3660,7 +3660,7 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>175</v>
+        <v>92.8</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -3668,7 +3668,7 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>181</v>
+        <v>143</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -3676,7 +3676,7 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>165</v>
+        <v>130</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -3684,7 +3684,7 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>165</v>
+        <v>141</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -3692,7 +3692,7 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>168</v>
+        <v>78.5</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -3700,7 +3700,7 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -3708,7 +3708,7 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>168</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -3716,7 +3716,7 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>196</v>
+        <v>78.5</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -3724,7 +3724,7 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>165</v>
+        <v>82.09999999999999</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -3732,7 +3732,7 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>162</v>
+        <v>141</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -3740,7 +3740,7 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>168</v>
+        <v>60.7</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -3748,7 +3748,7 @@
         <v>55</v>
       </c>
       <c r="B56">
-        <v>171</v>
+        <v>78.5</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -3756,7 +3756,7 @@
         <v>56</v>
       </c>
       <c r="B57">
-        <v>184</v>
+        <v>67.8</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -3764,7 +3764,7 @@
         <v>57</v>
       </c>
       <c r="B58">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -3772,7 +3772,7 @@
         <v>58</v>
       </c>
       <c r="B59">
-        <v>171</v>
+        <v>82.7</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -3780,7 +3780,7 @@
         <v>59</v>
       </c>
       <c r="B60">
-        <v>171</v>
+        <v>120</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -3788,7 +3788,7 @@
         <v>60</v>
       </c>
       <c r="B61">
-        <v>159</v>
+        <v>64.2</v>
       </c>
     </row>
   </sheetData>
@@ -3821,13 +3821,13 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -3835,13 +3835,13 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>-110393</v>
+        <v>66</v>
       </c>
       <c r="C3">
-        <v>-110393</v>
+        <v>49</v>
       </c>
       <c r="D3">
-        <v>-220786</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -3849,13 +3849,13 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C4">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -3863,13 +3863,13 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -3877,13 +3877,13 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C6">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -3891,13 +3891,13 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>-110393</v>
+        <v>140</v>
       </c>
       <c r="C7">
-        <v>-110393</v>
+        <v>148</v>
       </c>
       <c r="D7">
-        <v>-220786</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -3905,13 +3905,13 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C8">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -3919,13 +3919,13 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C9">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -3933,13 +3933,13 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C10">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -3947,13 +3947,13 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -3961,13 +3961,13 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>-110393</v>
+        <v>538</v>
       </c>
       <c r="D12">
-        <v>-220786</v>
+        <v>538</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -3975,13 +3975,13 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -3989,13 +3989,13 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D14">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -4003,13 +4003,13 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C15">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D15">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -4017,13 +4017,13 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -4031,13 +4031,13 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C17">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D17">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -4045,13 +4045,13 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C18">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -4059,13 +4059,13 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C19">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D19">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -4073,13 +4073,13 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C20">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D20">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -4087,13 +4087,13 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C21">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -4101,13 +4101,13 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C22">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -4115,13 +4115,13 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>-110393</v>
+        <v>94</v>
       </c>
       <c r="C23">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>-220786</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -4129,13 +4129,13 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C24">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -4143,13 +4143,13 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C25">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D25">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -4157,13 +4157,13 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C26">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -4171,13 +4171,13 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C27">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -4185,13 +4185,13 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C28">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -4199,13 +4199,13 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>-110393</v>
+        <v>367</v>
       </c>
       <c r="C29">
-        <v>-110393</v>
+        <v>259</v>
       </c>
       <c r="D29">
-        <v>-220786</v>
+        <v>626</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -4213,13 +4213,13 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C30">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D30">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -4227,13 +4227,13 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C31">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D31">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -4241,13 +4241,13 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C32">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D32">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -4255,13 +4255,13 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C33">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D33">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -4269,13 +4269,13 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C34">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D34">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -4283,13 +4283,13 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C35">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D35">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -4297,13 +4297,13 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C36">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D36">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -4311,13 +4311,13 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C37">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D37">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -4325,13 +4325,13 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C38">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D38">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -4339,13 +4339,13 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C39">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D39">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -4353,13 +4353,13 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C40">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D40">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -4367,13 +4367,13 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C41">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D41">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -4381,13 +4381,13 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C42">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -4395,13 +4395,13 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C43">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D43">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -4409,13 +4409,13 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C44">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D44">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -4423,13 +4423,13 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C45">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D45">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -4437,13 +4437,13 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C46">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D46">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -4451,13 +4451,13 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>-110393</v>
+        <v>140</v>
       </c>
       <c r="C47">
-        <v>-110393</v>
+        <v>116</v>
       </c>
       <c r="D47">
-        <v>-220786</v>
+        <v>256</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -4465,13 +4465,13 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C48">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D48">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -4479,13 +4479,13 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C49">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D49">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -4493,13 +4493,13 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C50">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D50">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -4507,13 +4507,13 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C51">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D51">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -4521,13 +4521,13 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>-110393</v>
+        <v>5323</v>
       </c>
       <c r="C52">
-        <v>-110393</v>
+        <v>1337</v>
       </c>
       <c r="D52">
-        <v>-220786</v>
+        <v>6660</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -4535,13 +4535,13 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C53">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D53">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -4549,13 +4549,13 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C54">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D54">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -4563,13 +4563,13 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>-110393</v>
+        <v>66</v>
       </c>
       <c r="C55">
-        <v>-110393</v>
+        <v>197</v>
       </c>
       <c r="D55">
-        <v>-220786</v>
+        <v>263</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -4577,13 +4577,13 @@
         <v>55</v>
       </c>
       <c r="B56">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C56">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D56">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -4591,13 +4591,13 @@
         <v>56</v>
       </c>
       <c r="B57">
-        <v>-110393</v>
+        <v>525</v>
       </c>
       <c r="C57">
-        <v>-110393</v>
+        <v>2960</v>
       </c>
       <c r="D57">
-        <v>-220786</v>
+        <v>3485</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -4605,13 +4605,13 @@
         <v>57</v>
       </c>
       <c r="B58">
-        <v>-110393</v>
+        <v>1558</v>
       </c>
       <c r="C58">
-        <v>-110393</v>
+        <v>10711</v>
       </c>
       <c r="D58">
-        <v>-220786</v>
+        <v>12269</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -4619,13 +4619,13 @@
         <v>58</v>
       </c>
       <c r="B59">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C59">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D59">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -4633,13 +4633,13 @@
         <v>59</v>
       </c>
       <c r="B60">
-        <v>-110393</v>
+        <v>433</v>
       </c>
       <c r="C60">
-        <v>-110393</v>
+        <v>748</v>
       </c>
       <c r="D60">
-        <v>-220786</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -4647,13 +4647,13 @@
         <v>60</v>
       </c>
       <c r="B61">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="C61">
-        <v>-110393</v>
+        <v>0</v>
       </c>
       <c r="D61">
-        <v>-220786</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4680,7 +4680,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>12.1</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -4688,7 +4688,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>12.1</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -4696,7 +4696,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>12.1</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -4704,7 +4704,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>12.1</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -4712,7 +4712,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>12.1</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -4720,7 +4720,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>12.6</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -4728,7 +4728,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -4736,7 +4736,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -4744,7 +4744,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4752,7 +4752,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -4760,7 +4760,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -4768,7 +4768,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -4776,7 +4776,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -4784,7 +4784,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -4792,7 +4792,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -4800,7 +4800,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -4808,7 +4808,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -4816,7 +4816,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -4824,7 +4824,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -4832,7 +4832,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -4840,7 +4840,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -4848,7 +4848,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -4856,7 +4856,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>12.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -4864,7 +4864,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>12.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -4872,7 +4872,7 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>12.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -4880,7 +4880,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>12.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -4888,7 +4888,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>12.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -4896,7 +4896,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>12.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -4904,7 +4904,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>12.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -4912,7 +4912,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>12.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -4920,7 +4920,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -4928,7 +4928,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>12.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -4936,7 +4936,7 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>12.1</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -4944,7 +4944,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>12.1</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -4952,7 +4952,7 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -4960,7 +4960,7 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -4968,7 +4968,7 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -4976,7 +4976,7 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -4984,7 +4984,7 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>12.2</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -4992,7 +4992,7 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>12.2</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -5000,7 +5000,7 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -5008,7 +5008,7 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -5016,7 +5016,7 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>12.2</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -5024,7 +5024,7 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -5032,7 +5032,7 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -5040,7 +5040,7 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -5048,7 +5048,7 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>12.1</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -5056,7 +5056,7 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>12.1</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -5064,7 +5064,7 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>12.1</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -5072,7 +5072,7 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>12.1</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -5080,7 +5080,7 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>12.1</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -5088,7 +5088,7 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>12.1</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -5096,7 +5096,7 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>12.1</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -5104,7 +5104,7 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>12.1</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -5112,7 +5112,7 @@
         <v>55</v>
       </c>
       <c r="B56">
-        <v>12.1</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -5120,7 +5120,7 @@
         <v>56</v>
       </c>
       <c r="B57">
-        <v>12.1</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -5128,7 +5128,7 @@
         <v>57</v>
       </c>
       <c r="B58">
-        <v>12.1</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -5136,7 +5136,7 @@
         <v>58</v>
       </c>
       <c r="B59">
-        <v>12.1</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -5144,7 +5144,7 @@
         <v>59</v>
       </c>
       <c r="B60">
-        <v>12.1</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -5152,7 +5152,7 @@
         <v>60</v>
       </c>
       <c r="B61">
-        <v>12.1</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -5179,7 +5179,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -5187,7 +5187,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -5195,7 +5195,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -5203,7 +5203,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -5211,7 +5211,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -5219,7 +5219,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -5227,7 +5227,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -5235,7 +5235,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -5243,7 +5243,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -5251,7 +5251,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -5259,7 +5259,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -5267,7 +5267,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -5275,7 +5275,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -5283,7 +5283,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -5291,7 +5291,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -5299,7 +5299,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -5307,7 +5307,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -5315,7 +5315,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -5323,7 +5323,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -5331,7 +5331,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -5339,7 +5339,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -5347,7 +5347,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -5355,7 +5355,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -5363,7 +5363,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -5371,7 +5371,7 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -5379,7 +5379,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -5387,7 +5387,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -5395,7 +5395,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -5403,7 +5403,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -5411,7 +5411,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -5419,7 +5419,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -5427,7 +5427,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -5435,7 +5435,7 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -5443,7 +5443,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -5451,7 +5451,7 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -5459,7 +5459,7 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -5467,7 +5467,7 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -5475,7 +5475,7 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -5483,7 +5483,7 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -5491,7 +5491,7 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -5499,7 +5499,7 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -5507,7 +5507,7 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -5515,7 +5515,7 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -5523,7 +5523,7 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -5531,7 +5531,7 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -5539,7 +5539,7 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -5547,7 +5547,7 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -5555,7 +5555,7 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -5563,7 +5563,7 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -5571,7 +5571,7 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -5579,7 +5579,7 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -5587,7 +5587,7 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -5595,7 +5595,7 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -5603,7 +5603,7 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -5611,7 +5611,7 @@
         <v>55</v>
       </c>
       <c r="B56">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -5619,7 +5619,7 @@
         <v>56</v>
       </c>
       <c r="B57">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -5627,7 +5627,7 @@
         <v>57</v>
       </c>
       <c r="B58">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -5635,7 +5635,7 @@
         <v>58</v>
       </c>
       <c r="B59">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -5643,7 +5643,7 @@
         <v>59</v>
       </c>
       <c r="B60">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -5651,7 +5651,7 @@
         <v>60</v>
       </c>
       <c r="B61">
-        <v>99</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>